<commit_message>
Markdown analysis query change to answer question 7 for visualization
</commit_message>
<xml_diff>
--- a/04_reporting_data/03_promotions/markdown_category_impact.xlsx
+++ b/04_reporting_data/03_promotions/markdown_category_impact.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/046ed6e1f1e0f6c8/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/046ed6e1f1e0f6c8/Desktop/projects/drivers_of_retail_sales_performance/04_reporting_data/03_promotions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF5186B2-0C89-43FC-B2F3-B9F169C96E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{DF5186B2-0C89-43FC-B2F3-B9F169C96E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97ADBF7A-D07B-4B52-A600-EA6749C1662F}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-795" windowWidth="29040" windowHeight="16440" xr2:uid="{B3D3CE06-7B46-478C-B5AF-42BA05C769AB}"/>
   </bookViews>
@@ -458,7 +458,8 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Consistent naming of the promotions reporting and visual workbooks
</commit_message>
<xml_diff>
--- a/04_reporting_data/03_promotions/markdown_category_impact.xlsx
+++ b/04_reporting_data/03_promotions/markdown_category_impact.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/046ed6e1f1e0f6c8/Desktop/projects/drivers_of_retail_sales_performance/04_reporting_data/03_promotions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{DF5186B2-0C89-43FC-B2F3-B9F169C96E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97ADBF7A-D07B-4B52-A600-EA6749C1662F}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{DF5186B2-0C89-43FC-B2F3-B9F169C96E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEC1459F-B3B7-4E00-9095-D6FE223902D2}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-795" windowWidth="29040" windowHeight="16440" xr2:uid="{B3D3CE06-7B46-478C-B5AF-42BA05C769AB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{B3D3CE06-7B46-478C-B5AF-42BA05C769AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,40 +41,40 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>avg_markdown1</t>
-  </si>
-  <si>
-    <t>avg_markdown2</t>
-  </si>
-  <si>
-    <t>avg_markdown3</t>
-  </si>
-  <si>
-    <t>avg_markdown4</t>
-  </si>
-  <si>
-    <t>avg_markdown5</t>
-  </si>
-  <si>
     <t>avg_weekly_sales</t>
   </si>
   <si>
-    <t>2590,07</t>
-  </si>
-  <si>
-    <t>879,97</t>
-  </si>
-  <si>
-    <t>468,09</t>
-  </si>
-  <si>
-    <t>1083,13</t>
-  </si>
-  <si>
-    <t>1662,77</t>
-  </si>
-  <si>
-    <t>15981,26</t>
+    <t>markdown_category</t>
+  </si>
+  <si>
+    <t>Markdown2</t>
+  </si>
+  <si>
+    <t>17052,9</t>
+  </si>
+  <si>
+    <t>Markdown4</t>
+  </si>
+  <si>
+    <t>17026,38</t>
+  </si>
+  <si>
+    <t>Markdown3</t>
+  </si>
+  <si>
+    <t>16736,55</t>
+  </si>
+  <si>
+    <t>Markdown1</t>
+  </si>
+  <si>
+    <t>16215,49</t>
+  </si>
+  <si>
+    <t>Markdown5</t>
+  </si>
+  <si>
+    <t>16177,02</t>
   </si>
 </sst>
 </file>
@@ -136,6 +136,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,50 +459,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43DD17E-9D44-4375-B7F9-CA667CF6A256}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add question 7 visual on promotion impact
</commit_message>
<xml_diff>
--- a/04_reporting_data/03_promotions/markdown_category_impact.xlsx
+++ b/04_reporting_data/03_promotions/markdown_category_impact.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/046ed6e1f1e0f6c8/Desktop/projects/drivers_of_retail_sales_performance/04_reporting_data/03_promotions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{DF5186B2-0C89-43FC-B2F3-B9F169C96E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEC1459F-B3B7-4E00-9095-D6FE223902D2}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{DF5186B2-0C89-43FC-B2F3-B9F169C96E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8908AB4F-F359-4FCE-BA6F-84E3C7C1EE17}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{B3D3CE06-7B46-478C-B5AF-42BA05C769AB}"/>
+    <workbookView minimized="1" xWindow="-26610" yWindow="1530" windowWidth="17280" windowHeight="9420" xr2:uid="{B3D3CE06-7B46-478C-B5AF-42BA05C769AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>avg_weekly_sales</t>
   </si>
@@ -50,31 +50,16 @@
     <t>Markdown2</t>
   </si>
   <si>
-    <t>17052,9</t>
-  </si>
-  <si>
     <t>Markdown4</t>
   </si>
   <si>
-    <t>17026,38</t>
-  </si>
-  <si>
     <t>Markdown3</t>
   </si>
   <si>
-    <t>16736,55</t>
-  </si>
-  <si>
     <t>Markdown1</t>
   </si>
   <si>
-    <t>16215,49</t>
-  </si>
-  <si>
     <t>Markdown5</t>
-  </si>
-  <si>
-    <t>16177,02</t>
   </si>
 </sst>
 </file>
@@ -463,7 +448,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -479,40 +465,40 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="B2">
+        <v>17052.900000000001</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>17026.38</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>16736.55</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>16215.49</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>16177.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>